<commit_message>
2026-27 schedules: TBA games for every bracket round (19 added)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QGTYUUYhY2XtyfLz2uEMC6
</commit_message>
<xml_diff>
--- a/Neural Network - Codex Optimized/2026-27 Schedule Screenshots/master_schedule.xlsx
+++ b/Neural Network - Codex Optimized/2026-27 Schedule Screenshots/master_schedule.xlsx
@@ -3728,7 +3728,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>10:00 AM</t>
+          <t>1:00 PM</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3821,12 +3821,12 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
+          <t>Feather River</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
           <t>San Jose</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>Feather River</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -4095,11 +4095,15 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>home</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
-      <c r="G84" t="inlineStr"/>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>@ San Jose City College</t>
+        </is>
+      </c>
       <c r="H84" t="inlineStr">
         <is>
           <t>Lassen + LA Trade Tech</t>
@@ -5517,12 +5521,12 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
+          <t>LA Trade Tech</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
           <t>San Jose</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>LA Trade Tech</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -20239,7 +20243,7 @@
       </c>
       <c r="E462" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>home</t>
         </is>
       </c>
       <c r="F462" t="inlineStr"/>

</xml_diff>

<commit_message>
FanMatch: bracket games linked to the games feeding them, one TBA row per game; team schedules show win/loss paths; SBVC bracket
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QGTYUUYhY2XtyfLz2uEMC6
</commit_message>
<xml_diff>
--- a/Neural Network - Codex Optimized/2026-27 Schedule Screenshots/master_schedule.xlsx
+++ b/Neural Network - Codex Optimized/2026-27 Schedule Screenshots/master_schedule.xlsx
@@ -7156,7 +7156,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>4:00 PM</t>
+          <t>3:30 PM</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -7364,17 +7364,17 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>5:30 PM</t>
+          <t>5:00 PM</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Chabot</t>
+          <t>San Joaquin Delta</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Siskiyous</t>
+          <t>Foothill</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
@@ -7385,12 +7385,12 @@
       <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr">
         <is>
-          <t>@ American River Tournament</t>
+          <t>San Mateo Fall Classic @ San Mateo</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>Chabot + Siskiyous</t>
+          <t>San Joaquin Delta + Foothill</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -7408,121 +7408,125 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
+          <t>5:30 PM</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Chabot</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Siskiyous</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr"/>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>@ American River Tournament</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>Chabot + Siskiyous</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>SCHEDULED</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-11-12</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
           <t>6:00 PM</t>
         </is>
       </c>
-      <c r="C162" t="inlineStr">
+      <c r="C163" t="inlineStr">
         <is>
           <t>Butte</t>
         </is>
       </c>
-      <c r="D162" t="inlineStr">
+      <c r="D163" t="inlineStr">
         <is>
           <t>Sierra</t>
         </is>
       </c>
-      <c r="E162" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="F162" t="inlineStr"/>
-      <c r="G162" t="inlineStr"/>
-      <c r="H162" t="inlineStr">
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr"/>
+      <c r="G163" t="inlineStr"/>
+      <c r="H163" t="inlineStr">
         <is>
           <t>Sierra + Butte</t>
         </is>
       </c>
-      <c r="I162" t="inlineStr">
-        <is>
-          <t>SCHEDULED</t>
-        </is>
-      </c>
-      <c r="J162" t="inlineStr"/>
-    </row>
-    <row r="163">
-      <c r="A163" s="2" t="inlineStr">
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>SCHEDULED</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
         <is>
           <t>2026-11-12</t>
         </is>
       </c>
-      <c r="B163" s="2" t="inlineStr">
+      <c r="B164" s="2" t="inlineStr">
         <is>
           <t>6:00 PM</t>
         </is>
       </c>
-      <c r="C163" s="2" t="inlineStr">
+      <c r="C164" s="2" t="inlineStr">
         <is>
           <t>Fresno</t>
         </is>
       </c>
-      <c r="D163" s="2" t="inlineStr">
+      <c r="D164" s="2" t="inlineStr">
         <is>
           <t>Contra Costa</t>
         </is>
       </c>
-      <c r="E163" s="2" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="F163" s="2" t="inlineStr"/>
-      <c r="G163" s="2" t="inlineStr"/>
-      <c r="H163" s="2" t="inlineStr">
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="F164" s="2" t="inlineStr"/>
+      <c r="G164" s="2" t="inlineStr"/>
+      <c r="H164" s="2" t="inlineStr">
         <is>
           <t>Contra Costa + Fresno</t>
         </is>
       </c>
-      <c r="I163" s="2" t="inlineStr">
-        <is>
-          <t>SCHEDULED</t>
-        </is>
-      </c>
-      <c r="J163" s="2" t="inlineStr">
+      <c r="I164" s="2" t="inlineStr">
+        <is>
+          <t>SCHEDULED</t>
+        </is>
+      </c>
+      <c r="J164" s="2" t="inlineStr">
         <is>
           <t>Moorpark opponent game</t>
         </is>
       </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t>2026-11-12</t>
-        </is>
-      </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>7:00 PM</t>
-        </is>
-      </c>
-      <c r="C164" t="inlineStr">
-        <is>
-          <t>Mt. San Antonio</t>
-        </is>
-      </c>
-      <c r="D164" t="inlineStr">
-        <is>
-          <t>Glendale</t>
-        </is>
-      </c>
-      <c r="E164" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="F164" t="inlineStr"/>
-      <c r="G164" t="inlineStr"/>
-      <c r="H164" t="inlineStr">
-        <is>
-          <t>Mt. San Antonio + Glendale</t>
-        </is>
-      </c>
-      <c r="I164" t="inlineStr">
-        <is>
-          <t>SCHEDULED</t>
-        </is>
-      </c>
-      <c r="J164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -7537,28 +7541,24 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>San Joaquin Delta</t>
+          <t>Mt. San Antonio</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Foothill</t>
+          <t>Glendale</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>home</t>
         </is>
       </c>
       <c r="F165" t="inlineStr"/>
-      <c r="G165" t="inlineStr">
-        <is>
-          <t>San Mateo Fall Classic @ San Mateo</t>
-        </is>
-      </c>
+      <c r="G165" t="inlineStr"/>
       <c r="H165" t="inlineStr">
         <is>
-          <t>San Joaquin Delta + Foothill</t>
+          <t>Mt. San Antonio + Glendale</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -8221,92 +8221,92 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" t="inlineStr">
+      <c r="A181" s="2" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="B181" t="inlineStr">
+      <c r="B181" s="2" t="inlineStr">
         <is>
           <t>5:30 PM</t>
         </is>
       </c>
-      <c r="C181" t="inlineStr">
+      <c r="C181" s="2" t="inlineStr">
+        <is>
+          <t>Feather River</t>
+        </is>
+      </c>
+      <c r="D181" s="2" t="inlineStr">
+        <is>
+          <t>Cuesta</t>
+        </is>
+      </c>
+      <c r="E181" s="2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="F181" s="2" t="inlineStr"/>
+      <c r="G181" s="2" t="inlineStr">
+        <is>
+          <t>@ American River College</t>
+        </is>
+      </c>
+      <c r="H181" s="2" t="inlineStr">
+        <is>
+          <t>Feather River + Cuesta</t>
+        </is>
+      </c>
+      <c r="I181" s="2" t="inlineStr">
+        <is>
+          <t>SCHEDULED</t>
+        </is>
+      </c>
+      <c r="J181" s="2" t="inlineStr">
+        <is>
+          <t>Moorpark opponent game</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-11-13</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>5:30 PM</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
         <is>
           <t>Modesto</t>
         </is>
       </c>
-      <c r="D181" t="inlineStr">
+      <c r="D182" t="inlineStr">
         <is>
           <t>West Valley</t>
         </is>
       </c>
-      <c r="E181" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="F181" t="inlineStr"/>
-      <c r="G181" t="inlineStr"/>
-      <c r="H181" t="inlineStr">
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>home</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr"/>
+      <c r="G182" t="inlineStr"/>
+      <c r="H182" t="inlineStr">
         <is>
           <t>Modesto + West Valley</t>
         </is>
       </c>
-      <c r="I181" t="inlineStr">
-        <is>
-          <t>SCHEDULED</t>
-        </is>
-      </c>
-      <c r="J181" t="inlineStr"/>
-    </row>
-    <row r="182">
-      <c r="A182" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-13</t>
-        </is>
-      </c>
-      <c r="B182" s="2" t="inlineStr">
-        <is>
-          <t>6:00 PM</t>
-        </is>
-      </c>
-      <c r="C182" s="2" t="inlineStr">
-        <is>
-          <t>Feather River</t>
-        </is>
-      </c>
-      <c r="D182" s="2" t="inlineStr">
-        <is>
-          <t>Cuesta</t>
-        </is>
-      </c>
-      <c r="E182" s="2" t="inlineStr">
-        <is>
-          <t>neutral</t>
-        </is>
-      </c>
-      <c r="F182" s="2" t="inlineStr"/>
-      <c r="G182" s="2" t="inlineStr">
-        <is>
-          <t>@ American River College</t>
-        </is>
-      </c>
-      <c r="H182" s="2" t="inlineStr">
-        <is>
-          <t>Feather River + Cuesta</t>
-        </is>
-      </c>
-      <c r="I182" s="2" t="inlineStr">
-        <is>
-          <t>SCHEDULED</t>
-        </is>
-      </c>
-      <c r="J182" s="2" t="inlineStr">
-        <is>
-          <t>Moorpark opponent game</t>
-        </is>
-      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>SCHEDULED</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
@@ -8536,7 +8536,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>8:00 PM</t>
+          <t>7:30 PM</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">

</xml_diff>